<commit_message>
last data palm biomass
</commit_message>
<xml_diff>
--- a/biomass_data_matinha_USP.xlsx
+++ b/biomass_data_matinha_USP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pedro M\Desktop\r_analizes\palms_biomass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F39C5E-58F8-4151-B205-DD7F52D88756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A037F694-6892-48E6-BA78-A75114FF971A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9F188378-987B-47FF-A329-9F0565C0E1BF}"/>
   </bookViews>
@@ -499,7 +499,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F475214B-53DA-49F0-A7EF-0FA49EC8C506}">
-  <dimension ref="A1:J2539"/>
+  <dimension ref="A1:J2686"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -59258,6 +59258,3387 @@
         <v>24</v>
       </c>
     </row>
+    <row r="2540" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2540">
+        <v>1</v>
+      </c>
+      <c r="B2540">
+        <v>6</v>
+      </c>
+      <c r="C2540">
+        <v>1</v>
+      </c>
+      <c r="D2540">
+        <v>5.8</v>
+      </c>
+      <c r="E2540">
+        <v>5.5</v>
+      </c>
+      <c r="F2540">
+        <v>3</v>
+      </c>
+      <c r="I2540" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2541" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2541">
+        <v>1</v>
+      </c>
+      <c r="B2541">
+        <v>6</v>
+      </c>
+      <c r="C2541">
+        <v>2</v>
+      </c>
+      <c r="D2541">
+        <v>11</v>
+      </c>
+      <c r="E2541">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="F2541">
+        <v>12</v>
+      </c>
+      <c r="I2541" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2542" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2542">
+        <v>1</v>
+      </c>
+      <c r="B2542">
+        <v>6</v>
+      </c>
+      <c r="C2542">
+        <v>3</v>
+      </c>
+      <c r="D2542">
+        <v>20.3</v>
+      </c>
+      <c r="E2542">
+        <v>16.5</v>
+      </c>
+      <c r="F2542">
+        <v>95</v>
+      </c>
+      <c r="I2542" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2543" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2543">
+        <v>1</v>
+      </c>
+      <c r="B2543">
+        <v>6</v>
+      </c>
+      <c r="C2543">
+        <v>4</v>
+      </c>
+      <c r="D2543">
+        <v>17.95</v>
+      </c>
+      <c r="E2543">
+        <v>12.5</v>
+      </c>
+      <c r="F2543">
+        <v>45</v>
+      </c>
+      <c r="I2543" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2544" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2544">
+        <v>1</v>
+      </c>
+      <c r="B2544">
+        <v>6</v>
+      </c>
+      <c r="C2544">
+        <v>5</v>
+      </c>
+      <c r="D2544">
+        <v>16.16</v>
+      </c>
+      <c r="E2544">
+        <v>14</v>
+      </c>
+      <c r="F2544">
+        <v>50</v>
+      </c>
+      <c r="I2544" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2545" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2545">
+        <v>1</v>
+      </c>
+      <c r="B2545">
+        <v>6</v>
+      </c>
+      <c r="C2545">
+        <v>6</v>
+      </c>
+      <c r="D2545">
+        <v>14.7</v>
+      </c>
+      <c r="E2545">
+        <v>17</v>
+      </c>
+      <c r="F2545">
+        <v>90</v>
+      </c>
+      <c r="I2545" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2546" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2546">
+        <v>1</v>
+      </c>
+      <c r="B2546">
+        <v>6</v>
+      </c>
+      <c r="C2546">
+        <v>7</v>
+      </c>
+      <c r="D2546">
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="E2546">
+        <v>16.5</v>
+      </c>
+      <c r="F2546">
+        <v>40</v>
+      </c>
+      <c r="I2546" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2547" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2547">
+        <v>1</v>
+      </c>
+      <c r="B2547">
+        <v>6</v>
+      </c>
+      <c r="C2547">
+        <v>8</v>
+      </c>
+      <c r="D2547">
+        <v>10.18</v>
+      </c>
+      <c r="E2547">
+        <v>11.5</v>
+      </c>
+      <c r="F2547">
+        <v>25</v>
+      </c>
+      <c r="I2547" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2548" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2548">
+        <v>1</v>
+      </c>
+      <c r="B2548">
+        <v>6</v>
+      </c>
+      <c r="C2548">
+        <v>9</v>
+      </c>
+      <c r="D2548">
+        <v>12.8</v>
+      </c>
+      <c r="E2548">
+        <v>16</v>
+      </c>
+      <c r="F2548">
+        <v>60</v>
+      </c>
+      <c r="I2548" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2549" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2549">
+        <v>1</v>
+      </c>
+      <c r="B2549">
+        <v>6</v>
+      </c>
+      <c r="C2549">
+        <v>10</v>
+      </c>
+      <c r="D2549">
+        <v>3.4</v>
+      </c>
+      <c r="E2549">
+        <v>9</v>
+      </c>
+      <c r="F2549">
+        <v>7</v>
+      </c>
+      <c r="I2549" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2550" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2550">
+        <v>1</v>
+      </c>
+      <c r="B2550">
+        <v>6</v>
+      </c>
+      <c r="C2550">
+        <v>11</v>
+      </c>
+      <c r="D2550">
+        <v>10.8</v>
+      </c>
+      <c r="E2550">
+        <v>16</v>
+      </c>
+      <c r="F2550">
+        <v>40</v>
+      </c>
+      <c r="I2550" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2551" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2551">
+        <v>1</v>
+      </c>
+      <c r="B2551">
+        <v>6</v>
+      </c>
+      <c r="C2551">
+        <v>12</v>
+      </c>
+      <c r="D2551">
+        <v>8.5</v>
+      </c>
+      <c r="E2551">
+        <v>17</v>
+      </c>
+      <c r="F2551">
+        <v>40</v>
+      </c>
+      <c r="I2551" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2552" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2552">
+        <v>1</v>
+      </c>
+      <c r="B2552">
+        <v>6</v>
+      </c>
+      <c r="C2552">
+        <v>13</v>
+      </c>
+      <c r="D2552">
+        <v>15.35</v>
+      </c>
+      <c r="E2552">
+        <v>18</v>
+      </c>
+      <c r="F2552">
+        <v>60</v>
+      </c>
+      <c r="I2552" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2553" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2553">
+        <v>1</v>
+      </c>
+      <c r="B2553">
+        <v>6</v>
+      </c>
+      <c r="C2553">
+        <v>14</v>
+      </c>
+      <c r="D2553">
+        <v>24.77</v>
+      </c>
+      <c r="E2553">
+        <v>14.5</v>
+      </c>
+      <c r="F2553">
+        <v>95</v>
+      </c>
+      <c r="I2553" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2554" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2554">
+        <v>1</v>
+      </c>
+      <c r="B2554">
+        <v>6</v>
+      </c>
+      <c r="C2554">
+        <v>15</v>
+      </c>
+      <c r="D2554">
+        <v>9.15</v>
+      </c>
+      <c r="E2554">
+        <v>10.5</v>
+      </c>
+      <c r="F2554">
+        <v>7</v>
+      </c>
+      <c r="I2554" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2555" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2555">
+        <v>1</v>
+      </c>
+      <c r="B2555">
+        <v>6</v>
+      </c>
+      <c r="C2555">
+        <v>16</v>
+      </c>
+      <c r="D2555">
+        <v>14.08</v>
+      </c>
+      <c r="E2555">
+        <v>12.5</v>
+      </c>
+      <c r="F2555">
+        <v>17</v>
+      </c>
+      <c r="I2555" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2556" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2556">
+        <v>1</v>
+      </c>
+      <c r="B2556">
+        <v>6</v>
+      </c>
+      <c r="C2556">
+        <v>17</v>
+      </c>
+      <c r="D2556">
+        <v>16.14</v>
+      </c>
+      <c r="E2556">
+        <v>16.5</v>
+      </c>
+      <c r="F2556">
+        <v>16</v>
+      </c>
+      <c r="I2556" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2557" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2557">
+        <v>1</v>
+      </c>
+      <c r="B2557">
+        <v>6</v>
+      </c>
+      <c r="C2557">
+        <v>18</v>
+      </c>
+      <c r="D2557">
+        <v>11.84</v>
+      </c>
+      <c r="E2557">
+        <v>9.5</v>
+      </c>
+      <c r="F2557">
+        <v>16</v>
+      </c>
+      <c r="I2557" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2558" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2558">
+        <v>1</v>
+      </c>
+      <c r="B2558">
+        <v>6</v>
+      </c>
+      <c r="C2558">
+        <v>19</v>
+      </c>
+      <c r="D2558">
+        <v>17.87</v>
+      </c>
+      <c r="E2558">
+        <v>10.5</v>
+      </c>
+      <c r="F2558">
+        <v>30</v>
+      </c>
+      <c r="I2558" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2559" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2559">
+        <v>1</v>
+      </c>
+      <c r="B2559">
+        <v>6</v>
+      </c>
+      <c r="C2559">
+        <v>20</v>
+      </c>
+      <c r="D2559">
+        <v>16.16</v>
+      </c>
+      <c r="E2559">
+        <v>9.5</v>
+      </c>
+      <c r="F2559">
+        <v>17</v>
+      </c>
+      <c r="I2559" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2560" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2560">
+        <v>1</v>
+      </c>
+      <c r="B2560">
+        <v>6</v>
+      </c>
+      <c r="C2560">
+        <v>21</v>
+      </c>
+      <c r="D2560">
+        <v>21.61</v>
+      </c>
+      <c r="E2560">
+        <v>16.5</v>
+      </c>
+      <c r="F2560">
+        <v>97</v>
+      </c>
+      <c r="I2560" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2561" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2561">
+        <v>1</v>
+      </c>
+      <c r="B2561">
+        <v>6</v>
+      </c>
+      <c r="C2561">
+        <v>22</v>
+      </c>
+      <c r="D2561">
+        <v>23.95</v>
+      </c>
+      <c r="E2561">
+        <v>22</v>
+      </c>
+      <c r="F2561">
+        <v>130</v>
+      </c>
+      <c r="I2561" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2562" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2562">
+        <v>1</v>
+      </c>
+      <c r="B2562">
+        <v>6</v>
+      </c>
+      <c r="C2562">
+        <v>23</v>
+      </c>
+      <c r="D2562">
+        <v>26.82</v>
+      </c>
+      <c r="E2562">
+        <v>13.5</v>
+      </c>
+      <c r="F2562">
+        <v>80</v>
+      </c>
+      <c r="I2562" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2563" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2563">
+        <v>1</v>
+      </c>
+      <c r="B2563">
+        <v>6</v>
+      </c>
+      <c r="C2563">
+        <v>24</v>
+      </c>
+      <c r="D2563">
+        <v>20.350000000000001</v>
+      </c>
+      <c r="E2563">
+        <v>19.5</v>
+      </c>
+      <c r="F2563">
+        <v>85</v>
+      </c>
+      <c r="I2563" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2564" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2564">
+        <v>1</v>
+      </c>
+      <c r="B2564">
+        <v>6</v>
+      </c>
+      <c r="C2564">
+        <v>25</v>
+      </c>
+      <c r="D2564">
+        <v>25.8</v>
+      </c>
+      <c r="E2564">
+        <v>22</v>
+      </c>
+      <c r="F2564">
+        <v>75</v>
+      </c>
+      <c r="I2564" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2565" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2565">
+        <v>1</v>
+      </c>
+      <c r="B2565">
+        <v>6</v>
+      </c>
+      <c r="C2565">
+        <v>26</v>
+      </c>
+      <c r="D2565">
+        <v>25</v>
+      </c>
+      <c r="E2565">
+        <v>18.5</v>
+      </c>
+      <c r="F2565">
+        <v>85</v>
+      </c>
+      <c r="I2565" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2566" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2566">
+        <v>1</v>
+      </c>
+      <c r="B2566">
+        <v>6</v>
+      </c>
+      <c r="C2566">
+        <v>27</v>
+      </c>
+      <c r="D2566">
+        <v>28.04</v>
+      </c>
+      <c r="E2566">
+        <v>19.5</v>
+      </c>
+      <c r="F2566">
+        <v>190</v>
+      </c>
+      <c r="I2566" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2567" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2567">
+        <v>1</v>
+      </c>
+      <c r="B2567">
+        <v>6</v>
+      </c>
+      <c r="C2567">
+        <v>28</v>
+      </c>
+      <c r="D2567">
+        <v>34.57</v>
+      </c>
+      <c r="E2567">
+        <v>28.5</v>
+      </c>
+      <c r="F2567">
+        <v>175</v>
+      </c>
+      <c r="I2567" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2568" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2568">
+        <v>1</v>
+      </c>
+      <c r="B2568">
+        <v>6</v>
+      </c>
+      <c r="C2568">
+        <v>29</v>
+      </c>
+      <c r="D2568">
+        <v>27.35</v>
+      </c>
+      <c r="E2568">
+        <v>25</v>
+      </c>
+      <c r="F2568">
+        <v>100</v>
+      </c>
+      <c r="I2568" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2569" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2569">
+        <v>1</v>
+      </c>
+      <c r="B2569">
+        <v>6</v>
+      </c>
+      <c r="C2569">
+        <v>30</v>
+      </c>
+      <c r="D2569">
+        <v>30.5</v>
+      </c>
+      <c r="E2569">
+        <v>27</v>
+      </c>
+      <c r="F2569">
+        <v>140</v>
+      </c>
+      <c r="I2569" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2570" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2570">
+        <v>1</v>
+      </c>
+      <c r="B2570">
+        <v>6</v>
+      </c>
+      <c r="C2570">
+        <v>31</v>
+      </c>
+      <c r="D2570">
+        <v>37.26</v>
+      </c>
+      <c r="E2570">
+        <v>30</v>
+      </c>
+      <c r="F2570">
+        <v>220</v>
+      </c>
+      <c r="I2570" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2571" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2571">
+        <v>1</v>
+      </c>
+      <c r="B2571">
+        <v>6</v>
+      </c>
+      <c r="C2571">
+        <v>32</v>
+      </c>
+      <c r="D2571">
+        <v>26.9</v>
+      </c>
+      <c r="E2571">
+        <v>22</v>
+      </c>
+      <c r="F2571">
+        <v>115</v>
+      </c>
+      <c r="I2571" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2572" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2572">
+        <v>1</v>
+      </c>
+      <c r="B2572">
+        <v>6</v>
+      </c>
+      <c r="C2572">
+        <v>33</v>
+      </c>
+      <c r="D2572">
+        <v>35</v>
+      </c>
+      <c r="E2572">
+        <v>33</v>
+      </c>
+      <c r="F2572">
+        <v>185</v>
+      </c>
+      <c r="I2572" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2573" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2573">
+        <v>1</v>
+      </c>
+      <c r="B2573">
+        <v>6</v>
+      </c>
+      <c r="C2573">
+        <v>34</v>
+      </c>
+      <c r="D2573">
+        <v>31.8</v>
+      </c>
+      <c r="E2573">
+        <v>28</v>
+      </c>
+      <c r="F2573">
+        <v>205</v>
+      </c>
+      <c r="I2573" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2574" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2574">
+        <v>1</v>
+      </c>
+      <c r="B2574">
+        <v>6</v>
+      </c>
+      <c r="C2574">
+        <v>35</v>
+      </c>
+      <c r="D2574">
+        <v>36.31</v>
+      </c>
+      <c r="E2574">
+        <v>27.5</v>
+      </c>
+      <c r="F2574">
+        <v>200</v>
+      </c>
+      <c r="I2574" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2575" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2575">
+        <v>1</v>
+      </c>
+      <c r="B2575">
+        <v>6</v>
+      </c>
+      <c r="C2575">
+        <v>36</v>
+      </c>
+      <c r="D2575">
+        <v>39.96</v>
+      </c>
+      <c r="E2575">
+        <v>36</v>
+      </c>
+      <c r="F2575">
+        <v>20</v>
+      </c>
+      <c r="I2575" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2576" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2576">
+        <v>1</v>
+      </c>
+      <c r="B2576">
+        <v>6</v>
+      </c>
+      <c r="C2576">
+        <v>37</v>
+      </c>
+      <c r="D2576">
+        <v>27.8</v>
+      </c>
+      <c r="E2576">
+        <v>28</v>
+      </c>
+      <c r="F2576">
+        <v>460</v>
+      </c>
+      <c r="I2576" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2577" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2577">
+        <v>1</v>
+      </c>
+      <c r="B2577">
+        <v>6</v>
+      </c>
+      <c r="C2577">
+        <v>38</v>
+      </c>
+      <c r="D2577">
+        <v>31.24</v>
+      </c>
+      <c r="E2577">
+        <v>28</v>
+      </c>
+      <c r="F2577">
+        <v>215</v>
+      </c>
+      <c r="I2577" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2578" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2578">
+        <v>1</v>
+      </c>
+      <c r="B2578">
+        <v>6</v>
+      </c>
+      <c r="C2578">
+        <v>39</v>
+      </c>
+      <c r="D2578">
+        <v>29.01</v>
+      </c>
+      <c r="E2578">
+        <v>27.5</v>
+      </c>
+      <c r="F2578">
+        <v>185</v>
+      </c>
+      <c r="I2578" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2579" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2579">
+        <v>1</v>
+      </c>
+      <c r="B2579">
+        <v>6</v>
+      </c>
+      <c r="C2579">
+        <v>40</v>
+      </c>
+      <c r="D2579">
+        <v>36.1</v>
+      </c>
+      <c r="E2579">
+        <v>30</v>
+      </c>
+      <c r="F2579">
+        <v>185</v>
+      </c>
+      <c r="I2579" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2580" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2580">
+        <v>1</v>
+      </c>
+      <c r="B2580">
+        <v>6</v>
+      </c>
+      <c r="C2580">
+        <v>41</v>
+      </c>
+      <c r="D2580">
+        <v>50</v>
+      </c>
+      <c r="E2580">
+        <v>36</v>
+      </c>
+      <c r="F2580">
+        <v>720</v>
+      </c>
+      <c r="I2580" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2581" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2581">
+        <v>1</v>
+      </c>
+      <c r="B2581">
+        <v>6</v>
+      </c>
+      <c r="C2581">
+        <v>42</v>
+      </c>
+      <c r="D2581">
+        <v>29.94</v>
+      </c>
+      <c r="E2581">
+        <v>29.5</v>
+      </c>
+      <c r="F2581">
+        <v>270</v>
+      </c>
+      <c r="I2581" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2582" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2582">
+        <v>1</v>
+      </c>
+      <c r="B2582">
+        <v>6</v>
+      </c>
+      <c r="C2582">
+        <v>43</v>
+      </c>
+      <c r="D2582">
+        <v>31.53</v>
+      </c>
+      <c r="E2582">
+        <v>24.5</v>
+      </c>
+      <c r="F2582">
+        <v>220</v>
+      </c>
+      <c r="I2582" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2583" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2583">
+        <v>1</v>
+      </c>
+      <c r="B2583">
+        <v>6</v>
+      </c>
+      <c r="C2583">
+        <v>44</v>
+      </c>
+      <c r="D2583">
+        <v>49.37</v>
+      </c>
+      <c r="E2583">
+        <v>95</v>
+      </c>
+      <c r="F2583">
+        <v>2290</v>
+      </c>
+      <c r="I2583" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2584" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2584">
+        <v>1</v>
+      </c>
+      <c r="B2584">
+        <v>8</v>
+      </c>
+      <c r="C2584">
+        <v>1</v>
+      </c>
+      <c r="D2584">
+        <v>10.48</v>
+      </c>
+      <c r="E2584">
+        <v>11</v>
+      </c>
+      <c r="F2584">
+        <v>13</v>
+      </c>
+      <c r="I2584" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2585" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2585">
+        <v>1</v>
+      </c>
+      <c r="B2585">
+        <v>8</v>
+      </c>
+      <c r="C2585">
+        <v>2</v>
+      </c>
+      <c r="D2585">
+        <v>12.51</v>
+      </c>
+      <c r="E2585">
+        <v>11</v>
+      </c>
+      <c r="F2585">
+        <v>17</v>
+      </c>
+      <c r="I2585" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2586" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2586">
+        <v>1</v>
+      </c>
+      <c r="B2586">
+        <v>8</v>
+      </c>
+      <c r="C2586">
+        <v>3</v>
+      </c>
+      <c r="D2586">
+        <v>5.61</v>
+      </c>
+      <c r="E2586">
+        <v>8.5</v>
+      </c>
+      <c r="F2586">
+        <v>7</v>
+      </c>
+      <c r="I2586" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2587" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2587">
+        <v>1</v>
+      </c>
+      <c r="B2587">
+        <v>8</v>
+      </c>
+      <c r="C2587">
+        <v>4</v>
+      </c>
+      <c r="D2587">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="E2587">
+        <v>10</v>
+      </c>
+      <c r="F2587">
+        <v>8</v>
+      </c>
+      <c r="I2587" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2588" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2588">
+        <v>1</v>
+      </c>
+      <c r="B2588">
+        <v>8</v>
+      </c>
+      <c r="C2588">
+        <v>5</v>
+      </c>
+      <c r="D2588">
+        <v>14.3</v>
+      </c>
+      <c r="E2588">
+        <v>19</v>
+      </c>
+      <c r="F2588">
+        <v>45</v>
+      </c>
+      <c r="I2588" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2589" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2589">
+        <v>1</v>
+      </c>
+      <c r="B2589">
+        <v>8</v>
+      </c>
+      <c r="C2589">
+        <v>6</v>
+      </c>
+      <c r="D2589">
+        <v>10.34</v>
+      </c>
+      <c r="E2589">
+        <v>8.5</v>
+      </c>
+      <c r="F2589">
+        <v>11</v>
+      </c>
+      <c r="I2589" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2590" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2590">
+        <v>1</v>
+      </c>
+      <c r="B2590">
+        <v>8</v>
+      </c>
+      <c r="C2590">
+        <v>7</v>
+      </c>
+      <c r="D2590">
+        <v>9.39</v>
+      </c>
+      <c r="E2590">
+        <v>10</v>
+      </c>
+      <c r="F2590">
+        <v>9</v>
+      </c>
+      <c r="I2590" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2591" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2591">
+        <v>1</v>
+      </c>
+      <c r="B2591">
+        <v>8</v>
+      </c>
+      <c r="C2591">
+        <v>8</v>
+      </c>
+      <c r="D2591">
+        <v>10.52</v>
+      </c>
+      <c r="E2591">
+        <v>9</v>
+      </c>
+      <c r="F2591">
+        <v>12</v>
+      </c>
+      <c r="I2591" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2592" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2592">
+        <v>1</v>
+      </c>
+      <c r="B2592">
+        <v>8</v>
+      </c>
+      <c r="C2592">
+        <v>9</v>
+      </c>
+      <c r="D2592">
+        <v>9.74</v>
+      </c>
+      <c r="E2592">
+        <v>9.5</v>
+      </c>
+      <c r="F2592">
+        <v>12</v>
+      </c>
+      <c r="I2592" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2593" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2593">
+        <v>1</v>
+      </c>
+      <c r="B2593">
+        <v>8</v>
+      </c>
+      <c r="C2593">
+        <v>10</v>
+      </c>
+      <c r="D2593">
+        <v>11.7</v>
+      </c>
+      <c r="E2593">
+        <v>10</v>
+      </c>
+      <c r="F2593">
+        <v>9</v>
+      </c>
+      <c r="I2593" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2594" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2594">
+        <v>1</v>
+      </c>
+      <c r="B2594">
+        <v>8</v>
+      </c>
+      <c r="C2594">
+        <v>11</v>
+      </c>
+      <c r="D2594">
+        <v>15.8</v>
+      </c>
+      <c r="E2594">
+        <v>13</v>
+      </c>
+      <c r="F2594">
+        <v>30</v>
+      </c>
+      <c r="I2594" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2595" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2595">
+        <v>1</v>
+      </c>
+      <c r="B2595">
+        <v>8</v>
+      </c>
+      <c r="C2595">
+        <v>12</v>
+      </c>
+      <c r="D2595">
+        <v>7.4</v>
+      </c>
+      <c r="E2595">
+        <v>8</v>
+      </c>
+      <c r="F2595">
+        <v>4</v>
+      </c>
+      <c r="I2595" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2596" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2596">
+        <v>1</v>
+      </c>
+      <c r="B2596">
+        <v>8</v>
+      </c>
+      <c r="C2596">
+        <v>13</v>
+      </c>
+      <c r="D2596">
+        <v>17.350000000000001</v>
+      </c>
+      <c r="E2596">
+        <v>12</v>
+      </c>
+      <c r="F2596">
+        <v>60</v>
+      </c>
+      <c r="I2596" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2597" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2597">
+        <v>1</v>
+      </c>
+      <c r="B2597">
+        <v>8</v>
+      </c>
+      <c r="C2597">
+        <v>14</v>
+      </c>
+      <c r="D2597">
+        <v>14.2</v>
+      </c>
+      <c r="E2597">
+        <v>15</v>
+      </c>
+      <c r="F2597">
+        <v>40</v>
+      </c>
+      <c r="I2597" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2598" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2598">
+        <v>1</v>
+      </c>
+      <c r="B2598">
+        <v>8</v>
+      </c>
+      <c r="C2598">
+        <v>15</v>
+      </c>
+      <c r="D2598">
+        <v>11.57</v>
+      </c>
+      <c r="E2598">
+        <v>15</v>
+      </c>
+      <c r="F2598">
+        <v>40</v>
+      </c>
+      <c r="I2598" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2599" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2599">
+        <v>1</v>
+      </c>
+      <c r="B2599">
+        <v>8</v>
+      </c>
+      <c r="C2599">
+        <v>16</v>
+      </c>
+      <c r="D2599">
+        <v>14.3</v>
+      </c>
+      <c r="E2599">
+        <v>11</v>
+      </c>
+      <c r="F2599">
+        <v>25</v>
+      </c>
+      <c r="I2599" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2600" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2600">
+        <v>1</v>
+      </c>
+      <c r="B2600">
+        <v>8</v>
+      </c>
+      <c r="C2600">
+        <v>17</v>
+      </c>
+      <c r="D2600">
+        <v>20.8</v>
+      </c>
+      <c r="E2600">
+        <v>19</v>
+      </c>
+      <c r="F2600">
+        <v>110</v>
+      </c>
+      <c r="I2600" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2601" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2601">
+        <v>1</v>
+      </c>
+      <c r="B2601">
+        <v>8</v>
+      </c>
+      <c r="C2601">
+        <v>18</v>
+      </c>
+      <c r="D2601">
+        <v>18.190000000000001</v>
+      </c>
+      <c r="E2601">
+        <v>14</v>
+      </c>
+      <c r="F2601">
+        <v>40</v>
+      </c>
+      <c r="I2601" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2602" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2602">
+        <v>1</v>
+      </c>
+      <c r="B2602">
+        <v>8</v>
+      </c>
+      <c r="C2602">
+        <v>19</v>
+      </c>
+      <c r="D2602">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="E2602">
+        <v>15</v>
+      </c>
+      <c r="F2602">
+        <v>50</v>
+      </c>
+      <c r="I2602" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2603" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2603">
+        <v>1</v>
+      </c>
+      <c r="B2603">
+        <v>8</v>
+      </c>
+      <c r="C2603">
+        <v>20</v>
+      </c>
+      <c r="D2603">
+        <v>26.21</v>
+      </c>
+      <c r="E2603">
+        <v>18</v>
+      </c>
+      <c r="F2603">
+        <v>115</v>
+      </c>
+      <c r="I2603" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2604" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2604">
+        <v>1</v>
+      </c>
+      <c r="B2604">
+        <v>8</v>
+      </c>
+      <c r="C2604">
+        <v>21</v>
+      </c>
+      <c r="D2604">
+        <v>21.4</v>
+      </c>
+      <c r="E2604">
+        <v>15.5</v>
+      </c>
+      <c r="F2604">
+        <v>110</v>
+      </c>
+      <c r="I2604" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2605" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2605">
+        <v>1</v>
+      </c>
+      <c r="B2605">
+        <v>8</v>
+      </c>
+      <c r="C2605">
+        <v>22</v>
+      </c>
+      <c r="D2605">
+        <v>17.440000000000001</v>
+      </c>
+      <c r="E2605">
+        <v>13.5</v>
+      </c>
+      <c r="F2605">
+        <v>45</v>
+      </c>
+      <c r="I2605" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2606" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2606">
+        <v>1</v>
+      </c>
+      <c r="B2606">
+        <v>8</v>
+      </c>
+      <c r="C2606">
+        <v>23</v>
+      </c>
+      <c r="D2606">
+        <v>12.47</v>
+      </c>
+      <c r="E2606">
+        <v>12.5</v>
+      </c>
+      <c r="F2606">
+        <v>22</v>
+      </c>
+      <c r="I2606" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2607" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2607">
+        <v>1</v>
+      </c>
+      <c r="B2607">
+        <v>8</v>
+      </c>
+      <c r="C2607">
+        <v>24</v>
+      </c>
+      <c r="D2607">
+        <v>14.93</v>
+      </c>
+      <c r="E2607">
+        <v>12.5</v>
+      </c>
+      <c r="F2607">
+        <v>35</v>
+      </c>
+      <c r="I2607" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2608" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2608">
+        <v>1</v>
+      </c>
+      <c r="B2608">
+        <v>8</v>
+      </c>
+      <c r="C2608">
+        <v>25</v>
+      </c>
+      <c r="D2608">
+        <v>18.13</v>
+      </c>
+      <c r="E2608">
+        <v>14.5</v>
+      </c>
+      <c r="F2608">
+        <v>45</v>
+      </c>
+      <c r="I2608" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2609" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2609">
+        <v>1</v>
+      </c>
+      <c r="B2609">
+        <v>8</v>
+      </c>
+      <c r="C2609">
+        <v>26</v>
+      </c>
+      <c r="D2609">
+        <v>19.149999999999999</v>
+      </c>
+      <c r="E2609">
+        <v>16.5</v>
+      </c>
+      <c r="F2609">
+        <v>55</v>
+      </c>
+      <c r="I2609" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2610" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2610">
+        <v>1</v>
+      </c>
+      <c r="B2610">
+        <v>8</v>
+      </c>
+      <c r="C2610">
+        <v>27</v>
+      </c>
+      <c r="D2610">
+        <v>18.37</v>
+      </c>
+      <c r="E2610">
+        <v>18</v>
+      </c>
+      <c r="F2610">
+        <v>55</v>
+      </c>
+      <c r="I2610" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2611" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2611">
+        <v>1</v>
+      </c>
+      <c r="B2611">
+        <v>8</v>
+      </c>
+      <c r="C2611">
+        <v>28</v>
+      </c>
+      <c r="D2611">
+        <v>26</v>
+      </c>
+      <c r="E2611">
+        <v>20.5</v>
+      </c>
+      <c r="F2611">
+        <v>135</v>
+      </c>
+      <c r="I2611" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2612" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2612">
+        <v>1</v>
+      </c>
+      <c r="B2612">
+        <v>8</v>
+      </c>
+      <c r="C2612">
+        <v>29</v>
+      </c>
+      <c r="D2612">
+        <v>20.54</v>
+      </c>
+      <c r="E2612">
+        <v>20.5</v>
+      </c>
+      <c r="F2612">
+        <v>95</v>
+      </c>
+      <c r="I2612" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2613" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2613">
+        <v>1</v>
+      </c>
+      <c r="B2613">
+        <v>8</v>
+      </c>
+      <c r="C2613">
+        <v>30</v>
+      </c>
+      <c r="D2613">
+        <v>15.26</v>
+      </c>
+      <c r="E2613">
+        <v>16</v>
+      </c>
+      <c r="F2613">
+        <v>60</v>
+      </c>
+      <c r="I2613" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2614" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2614">
+        <v>1</v>
+      </c>
+      <c r="B2614">
+        <v>8</v>
+      </c>
+      <c r="C2614">
+        <v>31</v>
+      </c>
+      <c r="D2614">
+        <v>20.09</v>
+      </c>
+      <c r="E2614">
+        <v>12.5</v>
+      </c>
+      <c r="F2614">
+        <v>80</v>
+      </c>
+      <c r="I2614" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2615" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2615">
+        <v>1</v>
+      </c>
+      <c r="B2615">
+        <v>8</v>
+      </c>
+      <c r="C2615">
+        <v>32</v>
+      </c>
+      <c r="D2615">
+        <v>22.05</v>
+      </c>
+      <c r="E2615">
+        <v>12.5</v>
+      </c>
+      <c r="F2615">
+        <v>45</v>
+      </c>
+      <c r="I2615" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2616" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2616">
+        <v>1</v>
+      </c>
+      <c r="B2616">
+        <v>8</v>
+      </c>
+      <c r="C2616">
+        <v>33</v>
+      </c>
+      <c r="D2616">
+        <v>32.58</v>
+      </c>
+      <c r="E2616">
+        <v>24.5</v>
+      </c>
+      <c r="F2616">
+        <v>230</v>
+      </c>
+      <c r="I2616" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2617" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2617">
+        <v>1</v>
+      </c>
+      <c r="B2617">
+        <v>8</v>
+      </c>
+      <c r="C2617">
+        <v>34</v>
+      </c>
+      <c r="D2617">
+        <v>28.06</v>
+      </c>
+      <c r="E2617">
+        <v>16.5</v>
+      </c>
+      <c r="F2617">
+        <v>195</v>
+      </c>
+      <c r="I2617" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2618" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2618">
+        <v>1</v>
+      </c>
+      <c r="B2618">
+        <v>8</v>
+      </c>
+      <c r="C2618">
+        <v>35</v>
+      </c>
+      <c r="D2618">
+        <v>28.14</v>
+      </c>
+      <c r="E2618">
+        <v>23.5</v>
+      </c>
+      <c r="F2618">
+        <v>205</v>
+      </c>
+      <c r="I2618" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2619" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2619">
+        <v>1</v>
+      </c>
+      <c r="B2619">
+        <v>8</v>
+      </c>
+      <c r="C2619">
+        <v>36</v>
+      </c>
+      <c r="D2619">
+        <v>30.45</v>
+      </c>
+      <c r="E2619">
+        <v>26</v>
+      </c>
+      <c r="F2619">
+        <v>235</v>
+      </c>
+      <c r="I2619" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2620" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2620">
+        <v>1</v>
+      </c>
+      <c r="B2620">
+        <v>8</v>
+      </c>
+      <c r="C2620">
+        <v>37</v>
+      </c>
+      <c r="D2620">
+        <v>34.22</v>
+      </c>
+      <c r="E2620">
+        <v>31</v>
+      </c>
+      <c r="F2620">
+        <v>295</v>
+      </c>
+      <c r="I2620" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2621" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2621">
+        <v>1</v>
+      </c>
+      <c r="B2621">
+        <v>8</v>
+      </c>
+      <c r="C2621">
+        <v>38</v>
+      </c>
+      <c r="D2621">
+        <v>27.98</v>
+      </c>
+      <c r="E2621">
+        <v>18.5</v>
+      </c>
+      <c r="F2621">
+        <v>195</v>
+      </c>
+      <c r="I2621" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2622" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2622">
+        <v>1</v>
+      </c>
+      <c r="B2622">
+        <v>8</v>
+      </c>
+      <c r="C2622">
+        <v>39</v>
+      </c>
+      <c r="D2622">
+        <v>24.59</v>
+      </c>
+      <c r="E2622">
+        <v>20</v>
+      </c>
+      <c r="F2622">
+        <v>125</v>
+      </c>
+      <c r="I2622" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2623" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2623">
+        <v>1</v>
+      </c>
+      <c r="B2623">
+        <v>8</v>
+      </c>
+      <c r="C2623">
+        <v>40</v>
+      </c>
+      <c r="D2623">
+        <v>26.25</v>
+      </c>
+      <c r="E2623">
+        <v>20</v>
+      </c>
+      <c r="F2623">
+        <v>150</v>
+      </c>
+      <c r="I2623" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2624" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2624">
+        <v>1</v>
+      </c>
+      <c r="B2624">
+        <v>8</v>
+      </c>
+      <c r="C2624">
+        <v>41</v>
+      </c>
+      <c r="D2624">
+        <v>25.29</v>
+      </c>
+      <c r="E2624">
+        <v>20</v>
+      </c>
+      <c r="F2624">
+        <v>145</v>
+      </c>
+      <c r="I2624" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2625" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2625">
+        <v>1</v>
+      </c>
+      <c r="B2625">
+        <v>8</v>
+      </c>
+      <c r="C2625">
+        <v>42</v>
+      </c>
+      <c r="D2625">
+        <v>34.39</v>
+      </c>
+      <c r="E2625">
+        <v>21</v>
+      </c>
+      <c r="F2625">
+        <v>205</v>
+      </c>
+      <c r="I2625" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2626" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2626">
+        <v>1</v>
+      </c>
+      <c r="B2626">
+        <v>8</v>
+      </c>
+      <c r="C2626">
+        <v>43</v>
+      </c>
+      <c r="D2626">
+        <v>23.28</v>
+      </c>
+      <c r="E2626">
+        <v>15</v>
+      </c>
+      <c r="F2626">
+        <v>100</v>
+      </c>
+      <c r="I2626" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2627" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2627">
+        <v>1</v>
+      </c>
+      <c r="B2627">
+        <v>8</v>
+      </c>
+      <c r="C2627">
+        <v>44</v>
+      </c>
+      <c r="D2627">
+        <v>28.13</v>
+      </c>
+      <c r="E2627">
+        <v>23.5</v>
+      </c>
+      <c r="F2627">
+        <v>160</v>
+      </c>
+      <c r="I2627" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2628" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2628">
+        <v>1</v>
+      </c>
+      <c r="B2628">
+        <v>8</v>
+      </c>
+      <c r="C2628">
+        <v>45</v>
+      </c>
+      <c r="D2628">
+        <v>17.239999999999998</v>
+      </c>
+      <c r="E2628">
+        <v>11</v>
+      </c>
+      <c r="F2628">
+        <v>40</v>
+      </c>
+      <c r="I2628" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2629" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2629">
+        <v>1</v>
+      </c>
+      <c r="B2629">
+        <v>8</v>
+      </c>
+      <c r="C2629">
+        <v>46</v>
+      </c>
+      <c r="D2629">
+        <v>17.77</v>
+      </c>
+      <c r="E2629">
+        <v>14.5</v>
+      </c>
+      <c r="F2629">
+        <v>55</v>
+      </c>
+      <c r="I2629" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2630" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2630">
+        <v>1</v>
+      </c>
+      <c r="B2630">
+        <v>8</v>
+      </c>
+      <c r="C2630">
+        <v>47</v>
+      </c>
+      <c r="D2630">
+        <v>24.66</v>
+      </c>
+      <c r="E2630">
+        <v>23.5</v>
+      </c>
+      <c r="F2630">
+        <v>210</v>
+      </c>
+      <c r="I2630" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2631" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2631">
+        <v>1</v>
+      </c>
+      <c r="B2631">
+        <v>8</v>
+      </c>
+      <c r="C2631">
+        <v>48</v>
+      </c>
+      <c r="D2631">
+        <v>19.7</v>
+      </c>
+      <c r="E2631">
+        <v>13</v>
+      </c>
+      <c r="F2631">
+        <v>50</v>
+      </c>
+      <c r="I2631" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2632" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2632">
+        <v>1</v>
+      </c>
+      <c r="B2632">
+        <v>8</v>
+      </c>
+      <c r="C2632">
+        <v>49</v>
+      </c>
+      <c r="D2632">
+        <v>11.94</v>
+      </c>
+      <c r="E2632">
+        <v>12</v>
+      </c>
+      <c r="F2632">
+        <v>22</v>
+      </c>
+      <c r="I2632" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2633" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2633">
+        <v>1</v>
+      </c>
+      <c r="B2633">
+        <v>8</v>
+      </c>
+      <c r="C2633">
+        <v>50</v>
+      </c>
+      <c r="D2633">
+        <v>50.03</v>
+      </c>
+      <c r="E2633">
+        <v>49</v>
+      </c>
+      <c r="F2633">
+        <v>920</v>
+      </c>
+      <c r="I2633" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2634" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2634">
+        <v>1</v>
+      </c>
+      <c r="B2634">
+        <v>8</v>
+      </c>
+      <c r="C2634">
+        <v>51</v>
+      </c>
+      <c r="D2634">
+        <v>40.450000000000003</v>
+      </c>
+      <c r="E2634">
+        <v>30</v>
+      </c>
+      <c r="F2634">
+        <v>460</v>
+      </c>
+      <c r="I2634" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2635" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2635">
+        <v>1</v>
+      </c>
+      <c r="B2635">
+        <v>8</v>
+      </c>
+      <c r="C2635">
+        <v>52</v>
+      </c>
+      <c r="D2635">
+        <v>39.630000000000003</v>
+      </c>
+      <c r="E2635">
+        <v>37</v>
+      </c>
+      <c r="F2635">
+        <v>510</v>
+      </c>
+      <c r="I2635" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2636" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2636">
+        <v>1</v>
+      </c>
+      <c r="B2636">
+        <v>8</v>
+      </c>
+      <c r="C2636">
+        <v>53</v>
+      </c>
+      <c r="D2636">
+        <v>45.72</v>
+      </c>
+      <c r="E2636">
+        <v>40</v>
+      </c>
+      <c r="F2636">
+        <v>700</v>
+      </c>
+      <c r="I2636" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2637" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2637">
+        <v>1</v>
+      </c>
+      <c r="B2637">
+        <v>8</v>
+      </c>
+      <c r="C2637">
+        <v>54</v>
+      </c>
+      <c r="D2637">
+        <v>39.33</v>
+      </c>
+      <c r="E2637">
+        <v>32</v>
+      </c>
+      <c r="F2637">
+        <v>460</v>
+      </c>
+      <c r="I2637" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2638" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2638">
+        <v>1</v>
+      </c>
+      <c r="B2638">
+        <v>8</v>
+      </c>
+      <c r="C2638">
+        <v>55</v>
+      </c>
+      <c r="D2638">
+        <v>35.6</v>
+      </c>
+      <c r="E2638">
+        <v>26</v>
+      </c>
+      <c r="F2638">
+        <v>330</v>
+      </c>
+      <c r="I2638" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2639" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2639">
+        <v>1</v>
+      </c>
+      <c r="B2639">
+        <v>8</v>
+      </c>
+      <c r="C2639">
+        <v>56</v>
+      </c>
+      <c r="D2639">
+        <v>35.46</v>
+      </c>
+      <c r="E2639">
+        <v>26.5</v>
+      </c>
+      <c r="F2639">
+        <v>350</v>
+      </c>
+      <c r="I2639" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2640" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2640">
+        <v>1</v>
+      </c>
+      <c r="B2640">
+        <v>8</v>
+      </c>
+      <c r="C2640">
+        <v>57</v>
+      </c>
+      <c r="D2640">
+        <v>38.06</v>
+      </c>
+      <c r="E2640">
+        <v>26</v>
+      </c>
+      <c r="F2640">
+        <v>380</v>
+      </c>
+      <c r="I2640" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2641" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2641">
+        <v>1</v>
+      </c>
+      <c r="B2641">
+        <v>8</v>
+      </c>
+      <c r="C2641">
+        <v>58</v>
+      </c>
+      <c r="D2641">
+        <v>40.049999999999997</v>
+      </c>
+      <c r="E2641">
+        <v>29</v>
+      </c>
+      <c r="F2641">
+        <v>350</v>
+      </c>
+      <c r="I2641" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2642" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2642">
+        <v>1</v>
+      </c>
+      <c r="B2642">
+        <v>8</v>
+      </c>
+      <c r="C2642">
+        <v>59</v>
+      </c>
+      <c r="D2642">
+        <v>35.14</v>
+      </c>
+      <c r="E2642">
+        <v>41</v>
+      </c>
+      <c r="F2642">
+        <v>620</v>
+      </c>
+      <c r="I2642" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2643" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2643">
+        <v>1</v>
+      </c>
+      <c r="B2643">
+        <v>8</v>
+      </c>
+      <c r="C2643">
+        <v>60</v>
+      </c>
+      <c r="D2643">
+        <v>27.05</v>
+      </c>
+      <c r="E2643">
+        <v>23</v>
+      </c>
+      <c r="F2643">
+        <v>200</v>
+      </c>
+      <c r="I2643" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2644" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2644">
+        <v>1</v>
+      </c>
+      <c r="B2644">
+        <v>8</v>
+      </c>
+      <c r="C2644">
+        <v>61</v>
+      </c>
+      <c r="D2644">
+        <v>42.65</v>
+      </c>
+      <c r="E2644">
+        <v>39</v>
+      </c>
+      <c r="F2644">
+        <v>570</v>
+      </c>
+      <c r="I2644" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2645" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2645">
+        <v>1</v>
+      </c>
+      <c r="B2645">
+        <v>8</v>
+      </c>
+      <c r="C2645">
+        <v>62</v>
+      </c>
+      <c r="D2645">
+        <v>42.54</v>
+      </c>
+      <c r="E2645">
+        <v>25.5</v>
+      </c>
+      <c r="F2645">
+        <v>480</v>
+      </c>
+      <c r="I2645" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2646" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2646">
+        <v>1</v>
+      </c>
+      <c r="B2646">
+        <v>8</v>
+      </c>
+      <c r="C2646">
+        <v>63</v>
+      </c>
+      <c r="D2646">
+        <v>51.33</v>
+      </c>
+      <c r="E2646">
+        <v>41</v>
+      </c>
+      <c r="F2646">
+        <v>730</v>
+      </c>
+      <c r="I2646" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2647" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2647">
+        <v>1</v>
+      </c>
+      <c r="B2647">
+        <v>8</v>
+      </c>
+      <c r="C2647">
+        <v>64</v>
+      </c>
+      <c r="D2647">
+        <v>52.25</v>
+      </c>
+      <c r="E2647">
+        <v>49</v>
+      </c>
+      <c r="F2647">
+        <v>1070</v>
+      </c>
+      <c r="I2647" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2648" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2648">
+        <v>1</v>
+      </c>
+      <c r="B2648">
+        <v>8</v>
+      </c>
+      <c r="C2648">
+        <v>65</v>
+      </c>
+      <c r="D2648">
+        <v>35.369999999999997</v>
+      </c>
+      <c r="E2648">
+        <v>28</v>
+      </c>
+      <c r="F2648">
+        <v>350</v>
+      </c>
+      <c r="I2648" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2649" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2649">
+        <v>1</v>
+      </c>
+      <c r="B2649">
+        <v>8</v>
+      </c>
+      <c r="C2649">
+        <v>66</v>
+      </c>
+      <c r="D2649">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="E2649">
+        <v>26.5</v>
+      </c>
+      <c r="F2649">
+        <v>400</v>
+      </c>
+      <c r="I2649" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2650" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2650">
+        <v>1</v>
+      </c>
+      <c r="B2650">
+        <v>8</v>
+      </c>
+      <c r="C2650">
+        <v>67</v>
+      </c>
+      <c r="D2650">
+        <v>54.32</v>
+      </c>
+      <c r="E2650">
+        <v>53.5</v>
+      </c>
+      <c r="F2650">
+        <v>1170</v>
+      </c>
+      <c r="I2650" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2651" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2651">
+        <v>1</v>
+      </c>
+      <c r="B2651">
+        <v>8</v>
+      </c>
+      <c r="C2651">
+        <v>68</v>
+      </c>
+      <c r="D2651">
+        <v>62.8</v>
+      </c>
+      <c r="E2651">
+        <v>100</v>
+      </c>
+      <c r="F2651">
+        <v>2780</v>
+      </c>
+      <c r="I2651" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2652" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2652">
+        <v>1</v>
+      </c>
+      <c r="B2652">
+        <v>8</v>
+      </c>
+      <c r="C2652">
+        <v>69</v>
+      </c>
+      <c r="D2652">
+        <v>51.71</v>
+      </c>
+      <c r="E2652">
+        <v>54.5</v>
+      </c>
+      <c r="F2652">
+        <v>1180</v>
+      </c>
+      <c r="I2652" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2653" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2653">
+        <v>1</v>
+      </c>
+      <c r="B2653">
+        <v>8</v>
+      </c>
+      <c r="C2653">
+        <v>70</v>
+      </c>
+      <c r="D2653">
+        <v>66.81</v>
+      </c>
+      <c r="E2653">
+        <v>68.5</v>
+      </c>
+      <c r="F2653">
+        <v>2100</v>
+      </c>
+      <c r="I2653" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2654" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2654">
+        <v>1</v>
+      </c>
+      <c r="B2654">
+        <v>8</v>
+      </c>
+      <c r="C2654">
+        <v>71</v>
+      </c>
+      <c r="D2654">
+        <v>59.73</v>
+      </c>
+      <c r="E2654">
+        <v>52.5</v>
+      </c>
+      <c r="F2654">
+        <v>1220</v>
+      </c>
+      <c r="I2654" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2655" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2655">
+        <v>1</v>
+      </c>
+      <c r="B2655">
+        <v>8</v>
+      </c>
+      <c r="C2655">
+        <v>72</v>
+      </c>
+      <c r="D2655">
+        <v>74.739999999999995</v>
+      </c>
+      <c r="E2655">
+        <v>146</v>
+      </c>
+      <c r="F2655">
+        <v>5420</v>
+      </c>
+      <c r="I2655" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2656" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2656">
+        <v>1</v>
+      </c>
+      <c r="B2656">
+        <v>7</v>
+      </c>
+      <c r="C2656">
+        <v>1</v>
+      </c>
+      <c r="D2656">
+        <v>5.81</v>
+      </c>
+      <c r="E2656">
+        <v>5.5</v>
+      </c>
+      <c r="F2656">
+        <v>2</v>
+      </c>
+      <c r="I2656" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2657" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2657">
+        <v>1</v>
+      </c>
+      <c r="B2657">
+        <v>7</v>
+      </c>
+      <c r="C2657">
+        <v>2</v>
+      </c>
+      <c r="D2657">
+        <v>9.57</v>
+      </c>
+      <c r="E2657">
+        <v>9</v>
+      </c>
+      <c r="F2657">
+        <v>7</v>
+      </c>
+      <c r="I2657" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2658" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2658">
+        <v>1</v>
+      </c>
+      <c r="B2658">
+        <v>7</v>
+      </c>
+      <c r="C2658">
+        <v>3</v>
+      </c>
+      <c r="D2658">
+        <v>17</v>
+      </c>
+      <c r="E2658">
+        <v>14</v>
+      </c>
+      <c r="F2658">
+        <v>25</v>
+      </c>
+      <c r="I2658" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2659" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2659">
+        <v>1</v>
+      </c>
+      <c r="B2659">
+        <v>7</v>
+      </c>
+      <c r="C2659">
+        <v>4</v>
+      </c>
+      <c r="D2659">
+        <v>12.79</v>
+      </c>
+      <c r="E2659">
+        <v>13</v>
+      </c>
+      <c r="F2659">
+        <v>16</v>
+      </c>
+      <c r="I2659" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2660" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2660">
+        <v>1</v>
+      </c>
+      <c r="B2660">
+        <v>7</v>
+      </c>
+      <c r="C2660">
+        <v>5</v>
+      </c>
+      <c r="D2660">
+        <v>11.36</v>
+      </c>
+      <c r="E2660">
+        <v>9</v>
+      </c>
+      <c r="F2660">
+        <v>14</v>
+      </c>
+      <c r="I2660" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2661" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2661">
+        <v>1</v>
+      </c>
+      <c r="B2661">
+        <v>7</v>
+      </c>
+      <c r="C2661">
+        <v>6</v>
+      </c>
+      <c r="D2661">
+        <v>9.59</v>
+      </c>
+      <c r="E2661">
+        <v>8.5</v>
+      </c>
+      <c r="F2661">
+        <v>6</v>
+      </c>
+      <c r="I2661" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2662" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2662">
+        <v>1</v>
+      </c>
+      <c r="B2662">
+        <v>7</v>
+      </c>
+      <c r="C2662">
+        <v>7</v>
+      </c>
+      <c r="D2662">
+        <v>12.19</v>
+      </c>
+      <c r="E2662">
+        <v>10</v>
+      </c>
+      <c r="F2662">
+        <v>7</v>
+      </c>
+      <c r="I2662" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2663" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2663">
+        <v>1</v>
+      </c>
+      <c r="B2663">
+        <v>7</v>
+      </c>
+      <c r="C2663">
+        <v>8</v>
+      </c>
+      <c r="D2663">
+        <v>17.440000000000001</v>
+      </c>
+      <c r="E2663">
+        <v>16.5</v>
+      </c>
+      <c r="F2663">
+        <v>55</v>
+      </c>
+      <c r="I2663" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2664" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2664">
+        <v>1</v>
+      </c>
+      <c r="B2664">
+        <v>7</v>
+      </c>
+      <c r="C2664">
+        <v>9</v>
+      </c>
+      <c r="D2664">
+        <v>14.1</v>
+      </c>
+      <c r="E2664">
+        <v>17</v>
+      </c>
+      <c r="F2664">
+        <v>40</v>
+      </c>
+      <c r="I2664" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2665" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2665">
+        <v>1</v>
+      </c>
+      <c r="B2665">
+        <v>7</v>
+      </c>
+      <c r="C2665">
+        <v>10</v>
+      </c>
+      <c r="D2665">
+        <v>18.440000000000001</v>
+      </c>
+      <c r="E2665">
+        <v>14</v>
+      </c>
+      <c r="F2665">
+        <v>45</v>
+      </c>
+      <c r="I2665" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2666" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2666">
+        <v>1</v>
+      </c>
+      <c r="B2666">
+        <v>7</v>
+      </c>
+      <c r="C2666">
+        <v>11</v>
+      </c>
+      <c r="D2666">
+        <v>16.579999999999998</v>
+      </c>
+      <c r="E2666">
+        <v>14.5</v>
+      </c>
+      <c r="F2666">
+        <v>45</v>
+      </c>
+      <c r="I2666" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2667" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2667">
+        <v>1</v>
+      </c>
+      <c r="B2667">
+        <v>7</v>
+      </c>
+      <c r="C2667">
+        <v>12</v>
+      </c>
+      <c r="D2667">
+        <v>17.61</v>
+      </c>
+      <c r="E2667">
+        <v>15</v>
+      </c>
+      <c r="F2667">
+        <v>50</v>
+      </c>
+      <c r="I2667" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2668" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2668">
+        <v>1</v>
+      </c>
+      <c r="B2668">
+        <v>7</v>
+      </c>
+      <c r="C2668">
+        <v>13</v>
+      </c>
+      <c r="D2668">
+        <v>26.02</v>
+      </c>
+      <c r="E2668">
+        <v>27</v>
+      </c>
+      <c r="F2668">
+        <v>180</v>
+      </c>
+      <c r="I2668" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2669" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2669">
+        <v>1</v>
+      </c>
+      <c r="B2669">
+        <v>7</v>
+      </c>
+      <c r="C2669">
+        <v>14</v>
+      </c>
+      <c r="D2669">
+        <v>25.55</v>
+      </c>
+      <c r="E2669">
+        <v>21</v>
+      </c>
+      <c r="F2669">
+        <v>110</v>
+      </c>
+      <c r="I2669" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2670" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2670">
+        <v>1</v>
+      </c>
+      <c r="B2670">
+        <v>7</v>
+      </c>
+      <c r="C2670">
+        <v>15</v>
+      </c>
+      <c r="D2670">
+        <v>22.02</v>
+      </c>
+      <c r="E2670">
+        <v>18</v>
+      </c>
+      <c r="F2670">
+        <v>210</v>
+      </c>
+      <c r="I2670" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2671" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2671">
+        <v>1</v>
+      </c>
+      <c r="B2671">
+        <v>7</v>
+      </c>
+      <c r="C2671">
+        <v>16</v>
+      </c>
+      <c r="D2671">
+        <v>23.53</v>
+      </c>
+      <c r="E2671">
+        <v>21</v>
+      </c>
+      <c r="F2671">
+        <v>125</v>
+      </c>
+      <c r="I2671" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2672" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2672">
+        <v>1</v>
+      </c>
+      <c r="B2672">
+        <v>7</v>
+      </c>
+      <c r="C2672">
+        <v>17</v>
+      </c>
+      <c r="D2672">
+        <v>28.96</v>
+      </c>
+      <c r="E2672">
+        <v>27.5</v>
+      </c>
+      <c r="F2672">
+        <v>245</v>
+      </c>
+      <c r="I2672" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2673" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2673">
+        <v>1</v>
+      </c>
+      <c r="B2673">
+        <v>7</v>
+      </c>
+      <c r="C2673">
+        <v>18</v>
+      </c>
+      <c r="D2673">
+        <v>23.55</v>
+      </c>
+      <c r="E2673">
+        <v>16.5</v>
+      </c>
+      <c r="F2673">
+        <v>95</v>
+      </c>
+      <c r="I2673" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2674" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2674">
+        <v>1</v>
+      </c>
+      <c r="B2674">
+        <v>7</v>
+      </c>
+      <c r="C2674">
+        <v>19</v>
+      </c>
+      <c r="D2674">
+        <v>22.06</v>
+      </c>
+      <c r="E2674">
+        <v>21.5</v>
+      </c>
+      <c r="F2674">
+        <v>125</v>
+      </c>
+      <c r="I2674" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2675" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2675">
+        <v>1</v>
+      </c>
+      <c r="B2675">
+        <v>7</v>
+      </c>
+      <c r="C2675">
+        <v>20</v>
+      </c>
+      <c r="D2675">
+        <v>36.659999999999997</v>
+      </c>
+      <c r="E2675">
+        <v>22.5</v>
+      </c>
+      <c r="F2675">
+        <v>205</v>
+      </c>
+      <c r="I2675" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2676" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2676">
+        <v>1</v>
+      </c>
+      <c r="B2676">
+        <v>7</v>
+      </c>
+      <c r="C2676">
+        <v>21</v>
+      </c>
+      <c r="D2676">
+        <v>24.87</v>
+      </c>
+      <c r="E2676">
+        <v>21</v>
+      </c>
+      <c r="F2676">
+        <v>160</v>
+      </c>
+      <c r="I2676" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2677" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2677">
+        <v>1</v>
+      </c>
+      <c r="B2677">
+        <v>7</v>
+      </c>
+      <c r="C2677">
+        <v>22</v>
+      </c>
+      <c r="D2677">
+        <v>46.51</v>
+      </c>
+      <c r="E2677">
+        <v>33</v>
+      </c>
+      <c r="F2677">
+        <v>550</v>
+      </c>
+      <c r="I2677" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2678" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2678">
+        <v>1</v>
+      </c>
+      <c r="B2678">
+        <v>7</v>
+      </c>
+      <c r="C2678">
+        <v>23</v>
+      </c>
+      <c r="D2678">
+        <v>32.770000000000003</v>
+      </c>
+      <c r="E2678">
+        <v>38.5</v>
+      </c>
+      <c r="F2678">
+        <v>380</v>
+      </c>
+      <c r="I2678" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2679" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2679">
+        <v>1</v>
+      </c>
+      <c r="B2679">
+        <v>7</v>
+      </c>
+      <c r="C2679">
+        <v>24</v>
+      </c>
+      <c r="D2679">
+        <v>40.15</v>
+      </c>
+      <c r="E2679">
+        <v>38.5</v>
+      </c>
+      <c r="F2679">
+        <v>590</v>
+      </c>
+      <c r="I2679" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2680" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2680">
+        <v>1</v>
+      </c>
+      <c r="B2680">
+        <v>7</v>
+      </c>
+      <c r="C2680">
+        <v>25</v>
+      </c>
+      <c r="D2680">
+        <v>40.96</v>
+      </c>
+      <c r="E2680">
+        <v>45.5</v>
+      </c>
+      <c r="F2680">
+        <v>790</v>
+      </c>
+      <c r="I2680" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2681" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2681">
+        <v>1</v>
+      </c>
+      <c r="B2681">
+        <v>7</v>
+      </c>
+      <c r="C2681">
+        <v>26</v>
+      </c>
+      <c r="D2681">
+        <v>54.53</v>
+      </c>
+      <c r="E2681">
+        <v>47.5</v>
+      </c>
+      <c r="F2681">
+        <v>1000</v>
+      </c>
+      <c r="I2681" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2682" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2682">
+        <v>1</v>
+      </c>
+      <c r="B2682">
+        <v>7</v>
+      </c>
+      <c r="C2682">
+        <v>27</v>
+      </c>
+      <c r="D2682">
+        <v>48.09</v>
+      </c>
+      <c r="E2682">
+        <v>50</v>
+      </c>
+      <c r="F2682">
+        <v>960</v>
+      </c>
+      <c r="I2682" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2683" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2683">
+        <v>1</v>
+      </c>
+      <c r="B2683">
+        <v>7</v>
+      </c>
+      <c r="C2683">
+        <v>28</v>
+      </c>
+      <c r="D2683">
+        <v>40.57</v>
+      </c>
+      <c r="E2683">
+        <v>38</v>
+      </c>
+      <c r="F2683">
+        <v>560</v>
+      </c>
+      <c r="I2683" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2684" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2684">
+        <v>1</v>
+      </c>
+      <c r="B2684">
+        <v>7</v>
+      </c>
+      <c r="C2684">
+        <v>29</v>
+      </c>
+      <c r="D2684">
+        <v>30.83</v>
+      </c>
+      <c r="E2684">
+        <v>27.5</v>
+      </c>
+      <c r="F2684">
+        <v>240</v>
+      </c>
+      <c r="I2684" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2685" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2685">
+        <v>1</v>
+      </c>
+      <c r="B2685">
+        <v>7</v>
+      </c>
+      <c r="C2685">
+        <v>30</v>
+      </c>
+      <c r="D2685">
+        <v>59.17</v>
+      </c>
+      <c r="E2685">
+        <v>41.5</v>
+      </c>
+      <c r="F2685">
+        <v>1010</v>
+      </c>
+      <c r="I2685" s="2">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="2686" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2686">
+        <v>1</v>
+      </c>
+      <c r="B2686">
+        <v>7</v>
+      </c>
+      <c r="C2686">
+        <v>31</v>
+      </c>
+      <c r="D2686">
+        <v>60.53</v>
+      </c>
+      <c r="E2686">
+        <v>110.5</v>
+      </c>
+      <c r="F2686">
+        <v>2940</v>
+      </c>
+      <c r="I2686" s="2">
+        <v>46115</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J2539" xr:uid="{F475214B-53DA-49F0-A7EF-0FA49EC8C506}"/>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>